<commit_message>
Alterações 18/06: Reorganização do código e dos arquivos, renomeando a pasta "exercicios" para "exercises" e movendo os arquivos de exercícios para lá. Além disso, foram feitas pequenas alterações em alguns arquivos de configuração e tradução.
</commit_message>
<xml_diff>
--- a/arquivos/tabelas_testes/sit_and_reach_test_julia.xlsx
+++ b/arquivos/tabelas_testes/sit_and_reach_test_julia.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3763,20 +3763,14 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
+      <c r="A116" t="n">
+        <v>22</v>
+      </c>
+      <c r="B116" t="n">
+        <v>165</v>
+      </c>
+      <c r="C116" t="n">
+        <v>63</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -3795,6 +3789,132 @@
       <c r="H116" t="inlineStr">
         <is>
           <t>left</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>22</v>
+      </c>
+      <c r="B117" t="n">
+        <v>165</v>
+      </c>
+      <c r="C117" t="n">
+        <v>63</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" t="n">
+        <v>-303.56</v>
+      </c>
+      <c r="G117" t="n">
+        <v>303.56</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>22</v>
+      </c>
+      <c r="B118" t="n">
+        <v>165</v>
+      </c>
+      <c r="C118" t="n">
+        <v>63</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>0</v>
+      </c>
+      <c r="F118" t="n">
+        <v>-297.02</v>
+      </c>
+      <c r="G118" t="n">
+        <v>297.02</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>22</v>
+      </c>
+      <c r="B119" t="n">
+        <v>165</v>
+      </c>
+      <c r="C119" t="n">
+        <v>63</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="G119" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="G120" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>right</t>
         </is>
       </c>
     </row>

</xml_diff>